<commit_message>
_src: scripts por etapa em cada bloco, nomes Bn-c/b/a e dicionário de nomes
Cada bloco de _src/ passa a ter collect/, build/, analise/, webscripts/,
logs/ e outros/. Os scripts viram Bn-<c|b|a>_<conteúdo>.py e gravam log em
logs/ (fora do git). Código compartilhado entre scripts foi para módulos
auxiliares (regic.py, CBOS em bases_comum.py), porque nome com hífen não é
importável. _src/dicionario.md reúne as convenções de nomes, atuais e
passadas, e regras novas para valores de colunas.
Pedido do autor, para separar etapas, encurtar nomes e guardar o histórico
das execuções.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/[B3] Contagem direta de ocupacao/B3_contagem_sorteio_visitas.xlsx
+++ b/dados/[B3] Contagem direta de ocupacao/B3_contagem_sorteio_visitas.xlsx
@@ -542,7 +542,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sorteio das visitas da contagem direta de ocupação (Bloco D)</t>
+          <t>Sorteio das visitas da contagem direta de ocupação (Bloco B3)</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• Os números aleatórios foram gerados com semente fixa (20260916) pelo script _src/[D] Contagem direta de ocupacao/build_contagem_sorteio.py e não devem ser editados.</t>
+          <t>• Os números aleatórios foram gerados com semente fixa (20260916) pelo script _src/[B3] Contagem direta de ocupacao/build/B3-b_contagem_sorteio.py e não devem ser editados.</t>
         </is>
       </c>
     </row>

</xml_diff>